<commit_message>
audit vs conditions: AppSource marketplace section in LR2-3, scenario matrix and section conclusions in LR7, stale DOSNYAT/price fixes in LR4, Excel template leftovers, refreshed instructions; rebuild
</commit_message>
<xml_diff>
--- a/ЛР2-3_Объем_рынка/Excel/ЛР2-3_4_цифровая_воронка_TableMind.xlsx
+++ b/ЛР2-3_Объем_рынка/Excel/ЛР2-3_4_цифровая_воронка_TableMind.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-continuation-57ce20\ЛР2-3_Объем_рынка\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-continuation-89518d\ЛР2-3_Объем_рынка\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8B42F9D-24C9-49DB-A1D3-51A9294F99FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42254B46-C511-4493-97D8-AEA622125D30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="458" windowWidth="12022" windowHeight="10972" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="311">
   <si>
     <t>Excel-шаблон оценки рынка через цифровую воронку</t>
   </si>
@@ -828,9 +828,6 @@
     <t>оценка охвата, клики, заявки</t>
   </si>
   <si>
-    <t>заполнить</t>
-  </si>
-  <si>
     <t>Фиксировать настройки аудитории.</t>
   </si>
   <si>
@@ -973,6 +970,12 @@
   </si>
   <si>
     <t>Рекламных кабинетов нет: использованы модельные показатели (допущение Д-33)</t>
+  </si>
+  <si>
+    <t>https://ads.google.com/ ; https://business.facebook.com/ (рекламные кабинеты не использовались, модельные показатели, Д-33)</t>
+  </si>
+  <si>
+    <t>perfectxl.com/pricing; arixcel.com/pricing; shortcut.ai/pricing; rows.com/pricing (страницы цен, 03.10.2026)</t>
   </si>
 </sst>
 </file>
@@ -2432,7 +2435,7 @@
         <v>243</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
@@ -2456,7 +2459,7 @@
         <v>243</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
@@ -2535,7 +2538,7 @@
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
     </row>
-    <row r="9" spans="1:10" ht="27">
+    <row r="9" spans="1:10" ht="108">
       <c r="A9" s="1" t="s">
         <v>259</v>
       </c>
@@ -2543,7 +2546,7 @@
         <v>260</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>261</v>
+        <v>309</v>
       </c>
       <c r="D9" s="8">
         <v>46298</v>
@@ -2552,22 +2555,22 @@
         <v>116</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
     </row>
-    <row r="10" spans="1:10" ht="40.5">
+    <row r="10" spans="1:10" ht="81">
       <c r="A10" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>264</v>
-      </c>
       <c r="C10" s="4" t="s">
-        <v>261</v>
+        <v>310</v>
       </c>
       <c r="D10" s="8">
         <v>46298</v>
@@ -2576,7 +2579,7 @@
         <v>116</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
@@ -3026,7 +3029,7 @@
         <v>65</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>66</v>
@@ -3050,7 +3053,7 @@
         <v>70</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>71</v>
@@ -3098,7 +3101,7 @@
         <v>79</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>80</v>
@@ -3122,7 +3125,7 @@
         <v>82</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>83</v>
@@ -3149,10 +3152,10 @@
         <v>19.43</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>271</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>272</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>88</v>
@@ -3173,7 +3176,7 @@
         <v>17.27</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>87</v>
@@ -3197,7 +3200,7 @@
         <v>20.29</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>87</v>
@@ -3224,7 +3227,7 @@
         <v>94</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>95</v>
@@ -3248,7 +3251,7 @@
         <v>94</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>97</v>
@@ -3302,7 +3305,7 @@
         <v>101</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>102</v>
@@ -3314,7 +3317,7 @@
         <v>104</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
@@ -3702,7 +3705,7 @@
         <v>111</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>138</v>
@@ -3711,7 +3714,7 @@
         <v>112</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>113</v>
@@ -3752,7 +3755,7 @@
         <v>116</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J4" s="1"/>
     </row>
@@ -3761,7 +3764,7 @@
         <v>115</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C5" s="6">
         <v>864031</v>
@@ -3784,7 +3787,7 @@
         <v>116</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J5" s="1"/>
     </row>
@@ -3816,7 +3819,7 @@
         <v>116</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J6" s="1"/>
     </row>
@@ -3825,7 +3828,7 @@
         <v>119</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C7" s="6">
         <v>153183</v>
@@ -3848,7 +3851,7 @@
         <v>116</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J7" s="1"/>
     </row>
@@ -3857,7 +3860,7 @@
         <v>118</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C8" s="6">
         <v>57025</v>
@@ -3880,13 +3883,13 @@
         <v>116</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J8" s="1"/>
     </row>
     <row r="9" spans="1:10" ht="40.5">
       <c r="A9" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>255</v>
@@ -3912,16 +3915,16 @@
         <v>116</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J9" s="1"/>
     </row>
     <row r="10" spans="1:10" ht="40.5">
       <c r="A10" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>282</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>283</v>
       </c>
       <c r="C10" s="6">
         <v>64643</v>
@@ -3944,7 +3947,7 @@
         <v>116</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J10" s="1"/>
     </row>
@@ -4447,10 +4450,10 @@
     </row>
     <row r="4" spans="1:10" ht="27">
       <c r="A4" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>286</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>287</v>
       </c>
       <c r="C4" s="6">
         <v>154111</v>
@@ -4476,15 +4479,15 @@
         <v>2447.7279898989395</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="27">
       <c r="A5" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>289</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>290</v>
       </c>
       <c r="C5" s="6">
         <v>35325</v>
@@ -4510,15 +4513,15 @@
         <v>2123.6922862200004</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="27">
       <c r="A6" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>291</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>292</v>
       </c>
       <c r="C6" s="6">
         <v>241737</v>
@@ -4544,15 +4547,15 @@
         <v>676.42506249093003</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="27">
       <c r="A7" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C7" s="6">
         <v>202178</v>
@@ -4578,15 +4581,15 @@
         <v>1682.1571013392797</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="27">
       <c r="A8" s="4" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C8" s="6">
         <v>14688</v>
@@ -4612,15 +4615,15 @@
         <v>1134.3446516736003</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="27">
       <c r="A9" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C9" s="6">
         <v>17824</v>
@@ -4646,15 +4649,15 @@
         <v>1347.2210340249599</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="27">
       <c r="A10" s="4" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C10" s="6">
         <v>292214</v>
@@ -4680,15 +4683,15 @@
         <v>1361.3857524383998</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="27">
       <c r="A11" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C11" s="6">
         <v>116617</v>
@@ -4714,15 +4717,15 @@
         <v>908.75977404814989</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="27">
       <c r="A12" s="4" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C12" s="6">
         <v>222359</v>
@@ -4748,15 +4751,15 @@
         <v>4611.0096106538404</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="27">
       <c r="A13" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C13" s="6">
         <v>701540</v>
@@ -4782,15 +4785,15 @@
         <v>983.61885120800002</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="27">
       <c r="A14" s="4" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C14" s="6">
         <v>1935</v>
@@ -4816,15 +4819,15 @@
         <v>167.14474519680002</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="27">
       <c r="A15" s="4" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C15" s="6">
         <v>5522</v>
@@ -4850,7 +4853,7 @@
         <v>95.013860958720002</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -5354,7 +5357,7 @@
     </row>
     <row r="4" spans="1:10" ht="67.5">
       <c r="A4" s="1" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B4" s="10">
         <f>'03_Конкуренты_SW'!C19</f>
@@ -5369,7 +5372,7 @@
         <v>158521.49098999999</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -7283,7 +7286,7 @@
         <v>201</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>202</v>
@@ -7308,7 +7311,7 @@
         <v>20.29</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>204</v>
@@ -7339,7 +7342,7 @@
         <v>405.79999999999995</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>207</v>
@@ -7355,7 +7358,7 @@
     </row>
     <row r="7" spans="1:10" ht="27">
       <c r="A7" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B7" s="7">
         <v>0.03</v>
@@ -7383,7 +7386,7 @@
     </row>
     <row r="8" spans="1:10" ht="27">
       <c r="A8" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B8" s="10">
         <f>B6*B7</f>
@@ -7398,7 +7401,7 @@
         <v>12.173999999999998</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>207</v>
@@ -7414,7 +7417,7 @@
     </row>
     <row r="9" spans="1:10" ht="27">
       <c r="A9" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B9" s="10">
         <f>B8*12</f>
@@ -7429,7 +7432,7 @@
         <v>146.08799999999997</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>207</v>
@@ -7953,7 +7956,7 @@
         <v>98.555981378302789</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>221</v>
@@ -7974,7 +7977,7 @@
         <v>1108.8261251768522</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>223</v>
@@ -7995,7 +7998,7 @@
         <v>8645.6860282789239</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>225</v>
@@ -8016,7 +8019,7 @@
         <v>5738.1751977902095</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>227</v>
@@ -8037,7 +8040,7 @@
         <v>1865.28</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>229</v>
@@ -8058,7 +8061,7 @@
         <v>55.958399999999997</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>231</v>

</xml_diff>